<commit_message>
fix: replace tilde range connectors with hyphens to prevent Markdown strikethrough
</commit_message>
<xml_diff>
--- a/backend/data/shard_dictionary.xlsx
+++ b/backend/data/shard_dictionary.xlsx
@@ -1734,7 +1734,7 @@
       </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
-          <t>Your Atomized Attributes are 2~20%stronger.</t>
+          <t>Your Atomized Attributes are 2~20% stronger.</t>
         </is>
       </c>
       <c r="M18" s="6" t="inlineStr">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="L48" s="6" t="inlineStr">
         <is>
-          <t>Grants 3~30%more Damage against Humanoid mobs.</t>
+          <t>Grants 3~30% more Damage against Humanoid mobs.</t>
         </is>
       </c>
       <c r="M48" s="6" t="inlineStr">
@@ -7656,7 +7656,7 @@
       </c>
       <c r="L112" s="6" t="inlineStr">
         <is>
-          <t>Your Essence Attributes are 2~20%stronger.</t>
+          <t>Your Essence Attributes are 2~20% stronger.</t>
         </is>
       </c>
       <c r="M112" s="6" t="inlineStr">
@@ -10932,7 +10932,7 @@
       </c>
       <c r="L164" s="6" t="inlineStr">
         <is>
-          <t>Your Resistance Attributes are 2~20%stronger.</t>
+          <t>Your Resistance Attributes are 2~20% stronger.</t>
         </is>
       </c>
       <c r="M164" s="6" t="inlineStr">
@@ -12188,7 +12188,7 @@
       </c>
       <c r="L184" s="6" t="inlineStr">
         <is>
-          <t>Your "Visitor" Attributes are 5~50%stronger.</t>
+          <t>Your "Visitor" Attributes are 5~50% stronger.</t>
         </is>
       </c>
       <c r="M184" s="6" t="inlineStr">
@@ -13700,7 +13700,7 @@
       </c>
       <c r="L208" s="6" t="inlineStr">
         <is>
-          <t>Grants 3~30%more Damage against Frozen mobs.</t>
+          <t>Grants 3~30% more Damage against Frozen mobs.</t>
         </is>
       </c>
       <c r="M208" s="6" t="inlineStr">
@@ -15149,7 +15149,7 @@
       </c>
       <c r="L231" s="6" t="inlineStr">
         <is>
-          <t>Grants 3~30%more Damage against Airborne mobs.</t>
+          <t>Grants 3~30% more Damage against Airborne mobs.</t>
         </is>
       </c>
       <c r="M231" s="6" t="inlineStr">
@@ -15716,7 +15716,7 @@
       </c>
       <c r="L240" s="6" t="inlineStr">
         <is>
-          <t>Grants 3~30%more Damage against Arcane mobs.</t>
+          <t>Grants 3~30% more Damage against Arcane mobs.</t>
         </is>
       </c>
       <c r="M240" s="6" t="inlineStr">
@@ -17039,7 +17039,7 @@
       </c>
       <c r="L261" s="6" t="inlineStr">
         <is>
-          <t>Grants 3~30%more Damage against Subterranean mobs.</t>
+          <t>Grants 3~30% more Damage against Subterranean mobs.</t>
         </is>
       </c>
       <c r="M261" s="6" t="inlineStr">
@@ -17858,7 +17858,7 @@
       </c>
       <c r="L274" s="6" t="inlineStr">
         <is>
-          <t>Grants 3~30%more Damage against Animal mobs.</t>
+          <t>Grants 3~30% more Damage against Animal mobs.</t>
         </is>
       </c>
       <c r="M274" s="6" t="inlineStr">
@@ -18047,7 +18047,7 @@
       </c>
       <c r="L277" s="6" t="inlineStr">
         <is>
-          <t>Grants 3~30%more Damage against Mythological mobs.</t>
+          <t>Grants 3~30% more Damage against Mythological mobs.</t>
         </is>
       </c>
       <c r="M277" s="6" t="inlineStr">
@@ -18677,7 +18677,7 @@
       </c>
       <c r="L287" s="6" t="inlineStr">
         <is>
-          <t>Grants 3~30%more Damage against Construct mobs.</t>
+          <t>Grants 3~30% more Damage against Construct mobs.</t>
         </is>
       </c>
       <c r="M287" s="6" t="inlineStr">
@@ -18740,7 +18740,7 @@
       </c>
       <c r="L288" s="6" t="inlineStr">
         <is>
-          <t>Grants 3~30%more Damage against Elusive mobs.</t>
+          <t>Grants 3~30% more Damage against Elusive mobs.</t>
         </is>
       </c>
       <c r="M288" s="6" t="inlineStr">
@@ -20567,7 +20567,7 @@
       </c>
       <c r="L317" s="6" t="inlineStr">
         <is>
-          <t>Your "Bucket" Attributes are 2~20%stronger.</t>
+          <t>Your "Bucket" Attributes are 2~20% stronger.</t>
         </is>
       </c>
       <c r="M317" s="6" t="inlineStr">

</xml_diff>